<commit_message>
Dataset: C1-BA evaluado por los tres expertos con notas idénticas (registradas una vez)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WQQKEDqM539xizMbxQojzM
</commit_message>
<xml_diff>
--- a/data/evaluai_dataset.xlsx
+++ b/data/evaluai_dataset.xlsx
@@ -109,7 +109,7 @@
     <t>Párrafo de conocimiento (no visible para el estudiante), versión detallada y simple</t>
   </si>
   <si>
-    <t>Notas (0-3) de los evaluadores humanos 1, 2 y 3. C1-BA tiene un único experto (grade_g2)</t>
+    <t>Notas (0-3) de los evaluadores humanos 1, 2 y 3. En C1-BA las tres notas coinciden y se registra una sola (grade_g2); las 3 respuestas de C1-BA excluidas por desacuerdo no se conservaron</t>
   </si>
   <si>
     <t>Puntaje (0-3) de una versión anterior del evaluador automático; solo disponible para C3</t>
@@ -3444,7 +3444,7 @@
     <t>human graders (2 of 3)</t>
   </si>
   <si>
-    <t>single expert</t>
+    <t>human graders (3 identical, recorded once)</t>
   </si>
   <si>
     <t>points</t>

</xml_diff>

<commit_message>
README del repositorio y de los datos en inglés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WQQKEDqM539xizMbxQojzM
</commit_message>
<xml_diff>
--- a/data/evaluai_dataset.xlsx
+++ b/data/evaluai_dataset.xlsx
@@ -88,64 +88,64 @@
     <t>score</t>
   </si>
   <si>
-    <t>Respuestas del curso Estructuras de Datos (ICI/ICD, PUCV) evaluadas por los tres expertos, antes y después del filtro de discrepancia. in_paper_290 marca las 287 usadas en el paper. Los id conservan la numeración original: los saltos corresponden a respuestas sin notas humanas completas, que se eliminaron</t>
-  </si>
-  <si>
-    <t>Identificador de la respuesta</t>
-  </si>
-  <si>
-    <t>Subconjunto según el paper: C3-S, C2-Smax, C2-hard, C1-BA</t>
-  </si>
-  <si>
-    <t>Nombre del subconjunto en el libro de trabajo original</t>
-  </si>
-  <si>
-    <t>Control del que proviene la respuesta (C1, C2, C3)</t>
-  </si>
-  <si>
-    <t>Identificador de la pregunta</t>
-  </si>
-  <si>
-    <t>Párrafo de conocimiento (no visible para el estudiante), versión detallada y simple</t>
-  </si>
-  <si>
-    <t>Notas (0-3) de los evaluadores humanos 1, 2 y 3. En C1-BA las tres notas coinciden (el libro original registra una sola, asignada a los tres); las 3 respuestas de C1-BA excluidas por desacuerdo no se conservaron</t>
-  </si>
-  <si>
-    <t>Puntaje (0-3) de una versión anterior del evaluador automático; solo disponible para C3</t>
-  </si>
-  <si>
-    <t>Cantidad de notas humanas y diferencia máxima entre ellas</t>
-  </si>
-  <si>
-    <t>Promedio de las notas humanas y puntaje de referencia (promedio redondeado; coincide con la moda cuando la diferencia es &lt;= 1)</t>
-  </si>
-  <si>
-    <t>La respuesta forma parte del dataset del paper (287 respuestas)</t>
-  </si>
-  <si>
-    <t>Motivo de exclusión de las respuestas que no forman parte del paper</t>
-  </si>
-  <si>
-    <t>Origen del puntaje de referencia</t>
-  </si>
-  <si>
-    <t>Respuestas de certámenes del curso de Optimización (2020-2024)</t>
-  </si>
-  <si>
-    <t>Certamen de origen</t>
-  </si>
-  <si>
-    <t>Respuesta correcta / pauta</t>
-  </si>
-  <si>
-    <t>Puntaje obtenido y puntaje máximo de la pregunta</t>
-  </si>
-  <si>
-    <t>Puntaje escalado a 0-3 y redondeado (round(points / max_points * 3))</t>
-  </si>
-  <si>
-    <t>Respuestas de niveles intermedios y completos usadas como ejemplos few-shot (no forman parte de DataStructures). Evaluadas por un único experto.</t>
+    <t>Responses from the Data Structures course (ICI/ICD, PUCV) graded by the three experts, before and after the disagreement filter. in_paper_290 marks the 287 responses used in the paper. The id column keeps the original numbering: gaps correspond to removed responses without complete human grades</t>
+  </si>
+  <si>
+    <t>Response identifier</t>
+  </si>
+  <si>
+    <t>Subset in the paper: C3-S, C2-Smax, C2-hard, C1-BA</t>
+  </si>
+  <si>
+    <t>Name of the subset in the original workbook</t>
+  </si>
+  <si>
+    <t>Assessment the response comes from (C1, C2, C3)</t>
+  </si>
+  <si>
+    <t>Question identifier</t>
+  </si>
+  <si>
+    <t>Knowledge paragraph (not shown to the student), detailed and simple versions</t>
+  </si>
+  <si>
+    <t>Grades (0-3) of human graders 1, 2 and 3. In C1-BA the three grades coincide (the original workbook records a single grade, assigned to the three graders); the 3 C1-BA responses excluded for disagreement were not kept</t>
+  </si>
+  <si>
+    <t>Score (0-3) given by an earlier version of the automatic grader; only available for C3</t>
+  </si>
+  <si>
+    <t>Number of human grades and maximum difference between them</t>
+  </si>
+  <si>
+    <t>Mean of the human grades and reference score (rounded mean; equal to the mode when the grades differ by at most 1)</t>
+  </si>
+  <si>
+    <t>The response is part of the paper dataset (287 responses)</t>
+  </si>
+  <si>
+    <t>Reason for excluding responses that are not part of the paper dataset</t>
+  </si>
+  <si>
+    <t>Source of the reference score</t>
+  </si>
+  <si>
+    <t>Exam responses from the Optimization course (2020-2024)</t>
+  </si>
+  <si>
+    <t>Exam the response comes from</t>
+  </si>
+  <si>
+    <t>Correct answer / grading guide</t>
+  </si>
+  <si>
+    <t>Points obtained and maximum points of the question</t>
+  </si>
+  <si>
+    <t>Score scaled to 0-3 and rounded (round(points / max_points * 3))</t>
+  </si>
+  <si>
+    <t>Intermediate and full-score responses used as few-shot examples (not part of DataStructures), graded by a single expert</t>
   </si>
   <si>
     <t>question</t>

</xml_diff>